<commit_message>
Daily EOD data and reports for 2026-08-25
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260825.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260825.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.825</v>
+        <v>1.9</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.025</v>
+        <v>0.05</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.35%</t>
+          <t>2.70%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>279555.33</v>
+        <v>291043.9</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-3829.53</v>
+        <v>7659.05</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.365</v>
+        <v>2.435</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.015</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.64%</t>
+          <t>3.62%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>165550</v>
+        <v>170450</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>1050</v>
+        <v>5950</v>
       </c>
     </row>
     <row r="6">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>67.86</v>
+        <v>67.61</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.74</v>
+        <v>0.49</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.10%</t>
+          <t>0.73%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>750870.9</v>
+        <v>748104.65</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8188.1</v>
+        <v>5421.85</v>
       </c>
     </row>
     <row r="8">
@@ -596,24 +596,24 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-0.003</v>
+        <v>0</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
         <v>44090</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0</v>
+        <v>132.27</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>-132.27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>158.51</v>
+        <v>157.45</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1.63</v>
+        <v>0.57</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.04%</t>
+          <t>0.36%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>1.025</v>
+        <v>1.04</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>0.015</v>
+        <v>0.03</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.49%</t>
+          <t>2.97%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>10250</v>
+        <v>10400</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>171.67</v>
+        <v>174.6</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2.56</v>
+        <v>5.49</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.51%</t>
+          <t>3.25%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>686680</v>
+        <v>698400</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>10240</v>
+        <v>21960</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0</v>
+        <v>0.27</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>-0.28</v>
+        <v>-0.01</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>-3.57%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0</v>
+        <v>5400</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>-5600</v>
+        <v>-200</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.115</v>
+        <v>0.112</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>4.55%</t>
+          <t>1.82%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1082.38</v>
+        <v>1054.14</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>47.06</v>
+        <v>18.82</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>33.75</v>
+        <v>34.06</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.01</v>
+        <v>0.32</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.03%</t>
+          <t>0.95%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>34.08</v>
+        <v>33.245</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.6</v>
+        <v>-0.235</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.79%</t>
+          <t>-0.70%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>43895.04</v>
+        <v>42819.56</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>772.8</v>
+        <v>-302.68</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1937883.65</v>
+        <v>1968404.52</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-58339.7</v>
+        <v>-27818.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>